<commit_message>
scenario_links_grdr_clean.xlsx save and temp files deletion
scenario_links_grdr_clean.xlsx save and temp files deletion
</commit_message>
<xml_diff>
--- a/hail/data/scenario_links_grdr_clean.xlsx
+++ b/hail/data/scenario_links_grdr_clean.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HOUJ\Downloads\Python_2\TIP\hail\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{06E0A39A-BC9C-4483-9F22-95D26C2DF2FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17183DCD-7B92-40B0-A00F-4351D432A7A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -545,7 +545,7 @@
   <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="53.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="8" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>